<commit_message>
chore(data): regenerate development coaching xlsx
</commit_message>
<xml_diff>
--- a/data/Development-Coaching-Tool.xlsx
+++ b/data/Development-Coaching-Tool.xlsx
@@ -451,7 +451,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-02-25T19:38:27.093Z</t>
+          <t>2026-02-25T19:58:06.007Z</t>
         </is>
       </c>
     </row>
@@ -475,7 +475,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026.02.25.90</t>
+          <t>2026.02.25.112</t>
         </is>
       </c>
     </row>
@@ -979,7 +979,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>{"generatedAt": "2026-02-25T19:38:27.093Z", "reason": "manual sync now", "sourceAppVersion": "2026.02.25.90", "weeklyData": {"2025-12-28|2026-01-03": {"employees": [{"name": "Marietta Bernal", "firstName": "Marietta", "scheduleAdherence": 97.67, "cxRepOverall": "", "fcr": "", "overallExperience": "", "transfers": 8.39, "transfersCount": 24, "aht": 404, "talkTime": 401, "acw": 0, "holdTime": 3, "reliability": 0, "overallSentiment": 83.2, "positiveWord": 77.3, "negativeWord": 78.4, "managingEmotions": 93.8, "surveyTotal": 0, "totalCalls": 286}, {"name": "Ekiecha Brabham", "firstName": "Ekiecha", "scheduleAdherence": 94.18, "cxRepOverall": "", "fcr": "", "overallExperience": "", "transfers": 6.94, "transfersCount": 12, "aht": 425, "talkTime": 251, "acw": 155, "holdTime": 18, "reliability": 0, "overallSentiment": 86.4, "positiveWord": 71.9, "negativeWord": 90.4, "managingEmotions": 97, "surveyTotal": 0, "totalCalls": 173}, {"name": "Caylie Chirumbolo", "firstName": "Caylie", "scheduleAdherence": 88.14, "cxRepOverall": 66.67, "fcr": 100, "overallExperience": 66.67, "transfers": 6.52, "transfersCount": 9, "aht": 468, "talkTime": 314, "acw": 128, "holdTime": 26, "reliability": 0.5, "overallSentiment": 92.8, "positiveWord": 90.3, "negativeWord": 91, "managingEmotions": 97, "surveyTotal": 3, "totalCalls": 138}, {"name": "Darryn Coley", "firstName": "Darryn", "scheduleAdherence": 89.41, "cxRepOverall": 0, "fcr": 100, "overallExperience": 0, "transfers": 8.84, "transfersCount": 16, "aht": 446, "talkTime": 248, "acw": 177, "holdTime": 21, "reliability": 0, "overallSentiment": 81.1, "positiveWord": 61.5, "negativeWord": 84.6, "managingEmotions": 97, "surveyTotal": 1, "totalCalls": 181}, {"name": "Ronda Colis", "firstName": "Ronda", "scheduleAdherence": 94.53, "cxRepOverall": "", "fcr": "", "overallExperience": "", "transfers": 5.68, "transfersCount": 5, "aht": 814, "talkTime": 591, "acw": 220, "holdTime": 3, "reliability": 0, "overallSentiment": 90.7, "positiveWord": 97.7, "negativeWord": 79.1, "managingEmotions": 95.3, "surveyTotal": 0, "totalCalls": 88}, {"name": "Taylor Colter", "firstName": "Taylor", "scheduleAdherence": 99.31, "cxRepOverall": "", "fcr": "", "overallExperience": "", "transfers": 0, "transfersCount": 0, "aht": 332, "talkTime": 315, "acw": 0, "holdTime": 17, "reliability": 0, "overallSentiment": 66.7, "positiveWord": "", "negativeWord": 100, "managingEmotions": 100, "surveyTotal": 0, "totalCalls": 72}, {"name": "Alyssa Dimes", "firstName": "Alyssa", "scheduleAdherence": 94.1, "cxRepOverall": "", "fcr": "", "overallExperience": "", "transfers": 5.1, "transfersCount": 8, "aht": 541, "talkTime": 378, "acw": 65, "holdTime": 98, "reliability": 0, "overallSentiment": 94.1, "positiveWord": 100, "negativeWord": 84.7, "managingEmotions": 97.5, "surveyTotal": 0, "totalCalls": 157}, {"name": "Trisha Erb", "firstName": "Trisha", "scheduleAdherence": 96.55, "cxRepOverall": "", "fcr": "", "overallExperience": "", "transfers": 10.43, "transfersCount": 12, "aht": 639, "talkTime": 466, "acw": 173, "holdTime": 0, "reliability": 0, "overallSentiment": 94.4, "positiveWord": 99.1, "negativeWord": 91.2, "managingEmotions": 92.9, "surveyTotal": 0, "totalCalls": 115}, {"name": "Angelina Fierro", "firstName": "Angelina", "scheduleAdherence": 93.43, "cxRepOverall": 100, "fcr": 100, "overallExperience": 100, "transfers": 6.72, "transfersCount": 9, "aht": 713, "talkTime": 545, "acw": 168, "holdTime": 0, "reliability": 0, "overallSentiment": 93.3, "positiveWord": 96.3, "negativeWord": 89.6, "managingEmotions": 94.1, "surveyTotal": 1, "totalCalls": 134}, {"name": "Jenifer Henson", "firstName": "Jenifer", "scheduleAdherence": 94, "cxRepOverall": "", "fcr": "", "overallExperience": "", "transfers": 7.65, "transfersCount": 13, "aht": 493, "talkTime": 478, "acw": 0, "holdTime": 15, "reliability": 0, "overallSentiment": 89.8, "positiveWord": 90.4, "negativeWord": 82.5, "managingEmotions": 96.4, "surveyTotal": 0, "totalCalls": 170}, {"name": "Oceane Ingram", "firstName": "Oceane", "scheduleAdherence": 86.78, "cxRepOverall": 100, "fcr": 100, "overallExperience": 100, "transfers": 12.31, "transfersCount": 16, "aht": 523, "talkTime": 271, "acw": 221, "holdTime": 32, "reliability": 0, "overallSentiment": 95.4, "positiveWord": 99.2, "negativeWord": 91.1, "managingEmotions": 95.9, "surveyTotal": 1, "totalCalls": 130}, {"name": "Precious Johnson", "firstName": "Precious", "scheduleAdherence": 93.88, "cxRepOverall": "", "fcr": "", "overallExperience": "", "transfers": 6.93, "transfersCount": 21, "aht": 371, "talkTime": 371, "acw": 1, "holdTime": 0, "reliability": 0, "overallSentiment": 93.4, "positiveWord": 97.7, "negativeWord": 85.7, "managingEmotions": 97, "surveyTotal": 0, "totalCalls": 303}, {"name": "Pamela Muhammad", "firstName": "Pamela", "scheduleAdherence": 94.43, "cxRepOverall": "", "fcr": "", "overallExperience": "", "transfers": 33.33, "transfersCount": 21, "aht": 782, "talkTime": 592, "acw": 171, "holdTime": 19, "reliability": 8.5, "overallSentiment": 85.7, "positiveWord": 73, "negativeWord": 87.3, "managingEmotions": 96.8, "surveyTotal": 0, "totalCalls": 63}, {"name": "Scoticia Osborne", "firstName": "Scoticia", "scheduleAdherence": 95.62, "cxRepOverall": "", "fcr": "", "overallExperience": "", "transfers": 3.85, "transfersCount": 5, "aht": 410, "talkTime": 364, "acw": 38, "holdTime": 8, "reliability": 0, "overallSentiment": 86.9, "positiveWord": 75.4, "negativeWord": 90, "managingEmotions": 95.4, "surveyTotal": 0, "totalCalls": 130}, {"name": "Teena Pokorski", "firstName": "Teena", "scheduleAdherence": 95.31, "cxRepOverall": 100, "fcr": 100, "overallExperience": 100, "transfers": 5.14, "transfersCount": 9, "aht": 514, "talkTime": 410, "acw": 98, "holdTime": 7, "reliability": 0, "overallSentiment": 94.3, "positiveWord": 98.3, "negativeWord": 88.5, "managingEmotions": 96, "surveyTotal": 2, "totalCalls": 175}], "metadata": {"startDate": "2025-12-28", "endDate": "2026-01-03", "label": "Week ending Jan 3, 2026", "periodType": "week", "yearEndTargetProfile": "auto", "yearEndReviewYear": "2026", "uploadedAt": "2026-02-21T04:27:22.786Z"}}, "2026-01-04|2026-01-10": {"employees": [{"name": "Ekiecha Brabham", "firstName": "Ekiecha", "scheduleAdherence": 89.85, "cxRepOverall": "", "fcr": "", "overallExperience": "", "transfers": 6.4, "transfersCount": 8, "aht": 455, "talkTime": 295, "acw": 150, "holdTime": 10, "reliability": 0, "overallSentiment": 81.6, "positiveWord": 69.5, "negativeWord": 80.5, "managingEmotions": 94.9, "surveyTotal": 0, "totalCalls": 125}, {"name": "Caylie Chirumbolo", "firstName": "Caylie", "scheduleAdherence": 84.5, "cxRepOverall": 0, "fcr": 0, "overallExperience": 0, "transfers": 9.78, "transfersCount": 18, "aht": 475, "talkTime": 321, "acw": 145, "holdTime": 10, "reliability": 0, "overallSentiment": 90.3, "positiveWord": 88.3, "negativeWord": 88.8, "managingEmotions": 93.9, "surveyTotal": 1, "totalCalls": 184}, {"name": "Darryn Coley", "firstName": "Darryn", "scheduleAdherence": 89.97, "cxRepOverall": "", "fcr": "", "overallExperience": "", "transfers": 11.21, "transfersCount": 13, "aht": 500, "talkTime": 355, "acw": 130, "holdTime": 16, "reliability": 0, "overallSentiment": 80.4, "positiveWord": 66.3, "negativeWord": 79.8, "managingEmotions": 95.2, "surveyTotal": 0, "totalCalls": 116}, {"name": "Ronda Colis", "firstName": "Ronda", "scheduleAdherence": 92.62, "cxRepOverall": "", "fcr": "", "overallExperience": "", "transfers": 4.49, "transfersCount": 4, "aht": 878, "talkTime": 651, "acw": 224, "holdTime": 2, "reliability": 0, "overallSentiment": 88.5, "positiveWord": 93.1, "negativeWord": 81.6, "managingEmotions": 90.8, "surveyTotal": 0, "totalCalls": 89}, {"name": "Taylor Colter", "firstName": "Taylor", "scheduleAdherence": 98.79, "cxRepOverall": "", "fcr": "", "overallExperience": "", "transfers": 0, "transfersCount": 0, "aht": 256, "talkTime": 248, "acw": 0, "holdTime": 7, "reliability": 0, "overallSentiment": 67.2, "positiveWord": 1.5, "negativeWord": 100, "managingEmotions": 100, "surveyTotal": 0, "totalCalls": 75}, {"name": "Alyssa Dimes", "firstName": "Alyssa", "scheduleAdherence": 94.28, "cxRepOverall": "", "fcr": "", "overallExperience": "", "transfers": 5.32, "transfersCount": 5, "aht": 628, "talkTime": 455, "acw": 69, "holdTime": 104, "reliability": 0, "overallSentiment": 92.2, "positiveWord": 97.9, "negativeWord": 85.1, "managingEmotions": 93.6, "surveyTotal": 0, "totalCalls": 94}, {"name": "Trisha Erb", "firstName": "Trisha", "scheduleAdherence": 95.22, "cxRepOverall": 100, "fcr": 100, "overallExperience": 100, "transfers": 10.18, "transfersCount": 17, "aht": 693, "talkTime": 479, "acw": 211, "holdTime": 3, "reliability": 0, "overallSentiment": 91.8, "positiveWord": 97, "negativeWord": 86.8, "managingEmotions": 91.6, "surveyTotal": 1, "totalCalls": 167}, {"name": "Angelina Fierro", "firstName": "Angelina", "scheduleAdherence": 90.95, "cxRepOverall": 100, "fcr": 100, "overallExperience": 100, "transfers": 12, "transfersCount": 18, "aht": 737, "talkTime": 562, "acw": 173, "holdTime": 2, "reliability": 0, "overallSentiment": 93.3, "positiveWord": 98, "negativeWord": 86, "managingEmotions": 96, "surveyTotal": 2, "totalCalls": 150}, {"name": "Jenifer Henson", "firstName": "Jenifer", "scheduleAdherence": 94.74, "cxRepOverall": 100, "fcr": 100, "overallExperience": 100, "transfers": 13.02, "transfersCount": 22, "aht": 491, "talkTime": 477, "acw": 0, "holdTime": 14, "reliability": 0, "overallSentiment": 87.8, "positiveWord": 89.2, "negativeWord": 77.8, "managingEmotions": 96.4, "surveyTotal": 1, "totalCalls": 169}, {"name": "Oceane Ingram", "firstName": "Oceane", "scheduleAdherence": 84.27, "cxRepOverall": 100, "fcr": 0, "overallExperience": 100, "transfers": 11.49, "transfersCount": 17, "aht": 551, "talkTime": 259, "acw": 246, "holdTime": 46, "reliability": 0, "overallSentiment": 95.6, "positiveWord": 98.6, "negativeWord": 93.7, "managingEmotions": 94.4, "surveyTotal": 1, "totalCalls": 148}, {"name": "Precious Johnson", "firstName": "Precious", "scheduleAdherence": 91.87, "cxRepOverall": 100, "fcr": 100, "overallExperience": 100, "transfers": 6.11, "transfersCount": 11, "aht": 430, "talkTime": 430, "acw": 0, "holdTime": 0, "reliability": 0, "overallSentiment": 94, "positiveWord": 99.4, "negativeWord": 87.2, "managingEmotions": 95.5, "surveyTotal": 3, "totalCalls": 180}, {"name": "Pamela Muhammad", "firstName": "Pamela", "scheduleAdherence": 98.66, "cxRepOverall": "", "fcr": "", "overallExperience": "", "transfers": 23.73, "transfersCount": 28, "aht": 694, "talkTime": 561, "acw": 93, "holdTime": 40, "reliability": 0, "overallSentiment": 90.5, "positiveWord": 84.5, "negativeWord": 90.5, "managingEmotions": 96.6, "surveyTotal": 0, "totalCalls": 118}, {"name": "Scoticia Osborne", "firstName": "Scoticia", "scheduleAdherence": 91.66, "cxRepOverall": 100, "fcr": 50, "overallExperience": 100, "transfers": 5, "transfersCount": 5, "aht": 451, "talkTime": 410, "acw": 38, "holdTime": 3, "reliability": 0, "overallSentiment": 89.1, "positiveWord": 90.5, "negativeWord": 83.2, "managingEmotions": 93.7, "surveyTotal": 2, "totalCalls": 100}, {"name": "Trevor Pedrowski", "firstName": "Trevor", "scheduleAdherence": 90.5, "cxRepOverall": 100, "fcr": "", "overallExperience": "", "transfers": 7.14, "transfersCount": 11, "aht": 470, "talkTime": 368, "acw": 91, "holdTime": 10, "reliability": 0, "overallSentiment": 84.1, "positiveWord": 75.5, "negativeWord": 81.6, "managingEmotions": 95.2, "surveyTotal": 0, "totalCalls": 154}, {"name": "Teena Pokorski", "firstName": "Teena", "scheduleAdherence": 92.96, "cxRepOverall": 100, "fcr": 50, "overallExperience": 100, "transfers": 7.94, "transfersCount": 17, "aht": 506, "talkTime": 387, "acw": 111, "holdTime": 8, "reliability": 0, "overallSentiment": 94.3, "positiveWord": 95.9, "negativeWord": 90.4, "managingEmotions": 96.8, "surveyTotal": 2, "totalCalls": 214}], "metadata": {"startDate": "2026-01-04", "endDate": "2026-01-10", "label": "Week ending Jan 10, 2026", "periodType": "week", "yearEndTargetProfile": "auto", "yearEndReviewYear": "2026", "uploadedAt": "2026-02-21T04:28:01.178Z"}}, "2026-01-11|2026-01-17": {"employees": [{"name": "Marietta Bernal", "firstName": "Marietta", "scheduleAdherence": 94.58, "cxRepOverall": 75, "fcr": 50, "overallExperience": 50, "transfers": 13.06, "transfersCount": 32, "aht": 434, "talkTime": 434, "acw": 0, "holdTime": 1, "reliability": 0, "overallSentiment": 80.5, "positiveWord": 70.2, "negativeWord": 76.9, "managingEmotions": 94.5, "surveyTotal": 4, "totalCalls": 245}, {"name": "Ekiecha Brabham", "firstName": "Ekiecha", "scheduleAdherence": 89.63, "cxRepOverall": 100, "fcr": 33.33, "overallExperience": 100, "transfers": 7.69, "transfersCount": 10, "aht": 417, "talkTime": 242, "acw": 146, "holdTime": 29, "reliability": 0, "overallSentiment": 85, "positiveWord": 68.3, "negativeWord": 89.2, "managingEmotions": 97.5, "surveyTotal": 3, "totalCalls": 130}, {"name": "Caylie Chirumbolo", "firstName": "Caylie", "scheduleAdherence": 91.44, "cxRepOverall": "", "fcr": "", "overallExperience": "", "transfers": 4.81, "transfersCount": 10, "aht": 460, "talkTime": 320, "acw": 124, "holdTime": 16, "reliability": 0.3, "overallSentiment": 92.6, "positiveWord": 94, "negativeWord": 85.4, "managingEmotions": 98.5, "surveyTotal": 0, "totalCalls": 208}, {"name": "Darryn Coley", "firstName": "Darryn", "scheduleAdherence": 80.17, "cxRepOverall": "", "fcr": "", "overallExperience": "", "transfers": 11.66, "transfersCount": 19, "aht": 517, "talkTime": 282, "acw": 201, "holdTime": 35, "reliability": 0.28, "overallSentiment": 83.3, "positiveWord": 72.3, "negativeWord": 82.4, "managingEmotions": 95.3, "surveyTotal": 0, "totalCalls": 163}, {"name": "Ronda Colis", "firstName": "Ronda", "scheduleAdherence": 93.85, "cxRepOverall": 100, "fcr": 100, "overallExperience": 50, "transfers": 5.15, "transfersCount": 5, "aht": 883, "talkTime": 650, "acw": 231, "holdTime": 2, "reliability": 0, "overallSentiment": 89.9, "positiveWord": 90.6, "negativeWord": 83.3, "managingEmotions": 95.8, "surveyTotal": 2, "totalCalls": 97}, {"name": "Taylor Colter", "firstName": "Taylor", "scheduleAdherence": 97.43, "cxRepOverall": "", "fcr": "", "overallExperience": "", "transfers": 0, "transfersCount": 0, "aht": 275, "talkTime": 268, "acw": 0, "holdTime": 6, "reliability": 0, "overallSentiment": 67.1, "positiveWord": 1.4, "negativeWord": 100, "managingEmotions": 100, "surveyTotal": 0, "totalCalls": 74}, {"name": "Alyssa Dimes", "firstName": "Alyssa", "scheduleAdherence": 88.67, "cxRepOverall": "", "fcr": "", "overallExperience": "", "transfers": 6.15, "transfersCount": 8, "aht": 678, "talkTime": 479, "acw": 64, "holdTime": 135, "reliability": 0, "overallSentiment": 94.7, "positiveWord": 96.9, "negativeWord": 90.1, "managingEmotions": 96.9, "surveyTotal": 0, "totalCalls": 130}, {"name": "Trisha Erb", "firstName": "Trisha", "scheduleAdherence": 90.06, "cxRepOverall": 100, "fcr": 0, "overallExperience": 100, "transfers": 7.04, "transfersCount": 5, "aht": 650, "talkTime": 412, "acw": 231, "holdTime": 7, "reliability": 0, "overallSentiment": 94.2, "positiveWord": 97.1, "negativeWord": 87, "managingEmotions": 98.6, "surveyTotal": 2, "totalCalls": 71}, {"name": "Angelina Fierro", "firstName": "Angelina", "scheduleAdherence": 83.46, "cxRepOverall": 100, "fcr": 100, "overallExperience": 100, "transfers": 3.67, "transfersCount": 4, "aht": 657, "talkTime": 486, "acw": 167, "holdTime": 4, "reliability": 0, "overallSentiment": 91.7, "positiveWord": 95.4, "negativeWord": 85.3, "managingEmotions": 94.5, "surveyTotal": 1, "totalCalls": 109}, {"name": "Jenifer Henson", "firstName": "Jenifer", "scheduleAdherence": 82.85, "cxRepOverall": 100, "fcr": 100, "overallExperience": 0, "transfers": 7.96, "transfersCount": 9, "aht": 535, "talkTime": 515, "acw": 0, "holdTime": 20, "reliability": 0, "overallSentiment": 89.6, "positiveWord": 93.8, "negativeWord": 83, "managingEmotions": 92, "surveyTotal": 1, "totalCalls": 113}, {"name": "Precious Johnson", "firstName": "Precious", "scheduleAdherence": 80.67, "cxRepOverall": 100, "fcr": 33.33, "overallExperience": 100, "transfers": 6.67, "transfersCount": 10, "aht": 392, "talkTime": 392, "acw": 0, "holdTime": 0, "reliability": 0, "overallSentiment": 93.8, "positiveWord": 99.3, "negativeWord": 84.1, "managingEmotions": 97.9, "surveyTotal": 3, "totalCalls": 150}, {"name": "Pamela Muhammad", "firstName": "Pamela", "scheduleAdherence": 95.42, "cxRepOverall": 50, "fcr": 0, "overallExperience": 50, "transfers": 32.82, "transfersCount": 86, "aht": 493, "talkTime": 392, "acw": 79, "holdTime": 22, "reliability": 0, "overallSentiment": 84.6, "positiveWord": 65.4, "negativeWord": 91.7, "managingEmotions": 96.9, "surveyTotal": 2, "totalCalls": 262}, {"name": "Scoticia Osborne", "firstName": "Scoticia", "scheduleAdherence": 90.78, "cxRepOverall": 100, "fcr": 100, "overallExperience": 100, "transfers": 7.69, "transfersCount": 14, "aht": 474, "talkTime": 433, "acw": 41, "holdTime": 0, "reliability": 0.3, "overallSentiment": 91.3, "positiveWord": 90, "negativeWord": 86.1, "managingEmotions": 97.8, "surveyTotal": 1, "totalCalls": 182}, {"name": "Trevor Pedrowski", "firstName": "Trevor", "scheduleAdherence": 86.16, "cxRepOverall": "", "fcr": "", "overallExperience": "", "transfers": 8.81, "transfersCount": 14, "aht": 467, "talkTime": 357, "acw": 89, "holdTime": 22, "reliability": 0, "overallSentiment": 79.3, "positiveWord": 66.4, "negativeWord": 79.3, "managingEmotions": 92.1, "surveyTotal": 0, "totalCalls": 159}, {"name": "Teena Pokorski", "firstName": "Teena", "scheduleAdherence": 94.71, "cxRepOverall": 100, "fcr": 100, "overallExperience": 100, "transfers": 8.26, "transfersCount": 18, "aht": 498, "talkTime": 368, "acw": 122, "holdTime": 8, "reliability": 0, "overallSentiment": 94.7, "positiveWord": 96.8, "negativeWord": 90.5, "managingEmotions": 96.8, "surveyTotal": 5, "totalCalls": 218}], "metadata": {"startDate": "2026-01-11", "endDate": "2026-01-17", "label": "Week ending Jan 17, 2026", "periodType": "week", "yearEndTargetProfile": "auto", "yearEndReviewYear": "2026", "uploadedAt": "2026-02-21T04:29:28.383Z"}}, "2026-01-18|2026-01-24": {"employees": [{"name": "Marietta Bernal", "firstName": "Marietta", "scheduleAdherence": 94.58, "cxRepOverall": 75, "fcr": 50, "overallExperience": 50, "transfers": 13.06, "transfersCount": 32, "aht": 434, "talkTime": 434, "acw": 0, "holdTime": 1, "reliability": 0, "overallSentiment": 80.5, "positiveWord": 70.2, "negativeWord": 76.9, "managingEmotions": 94.5, "surveyTotal": 4, "totalCalls": 245}, {"name": "Ekiecha Brabham", "firstName": "Ekiecha", "scheduleAdherence": 89.63, "cxRepOverall": 100, "fcr": 33.33, "overallExperience": 100, "transfers": 7.69, "transfersCount": 10, "aht": 417, "talkTime": 242, "acw": 146, "holdTime": 29, "reliability": 0, "overallSentiment": 85, "positiveWord": 68.3, "negativeWord": 89.2, "managingEmotions": 97.5, "surveyTotal": 3, "totalCalls": 130}, {"name": "Caylie Chirumbolo", "firstName": "Caylie", "scheduleAdherence": 91.44, "cxRepOverall": "", "fcr": "", "overallExperience": "", "transfers": 4.81, "transfersCount": 10, "aht": 460, "talkTime": 320, "acw": 124, "holdTime": 16, "reliability": 0.3, "overallSentiment": 92.6, "positiveWord": 94, "negativeWord": 85.4, "managingEmotions": 98.5, "surveyTotal": 0, "totalCalls": 208}, {"name": "Darryn Coley", "firstName": "Darryn", "scheduleAdherence": 80.17, "cxRepOverall": "", "fcr": "", "overallExperience": "", "transfers": 11.66, "transfersCount": 19, "aht": 517, "talkTime": 282, "acw": 201, "holdTime": 35, "reliability": 0.28, "overallSentiment": 83.3, "positiveWord": 72.3, "negativeWord": 82.4, "managingEmotions": 95.3, "surveyTotal": 0, "totalCalls": 163}, {"name": "Ronda Colis", "firstName": "Ronda", "scheduleAdherence": 93.85, "cxRepOverall": 100, "fcr": 100, "overallExperience": 50, "transfers": 5.15, "transfersCount": 5, "aht": 883, "talkTime": 650, "acw": 231, "holdTime": 2, "reliability": 0, "overallSentiment": 89.9, "positiveWord": 90.6, "negativeWord": 83.3, "managingEmotions": 95.8, "surveyTotal": 2, "totalCalls": 97}, {"name": "Taylor Colter", "firstName": "Taylor", "scheduleAdherence": 97.43, "cxRepOverall": "", "fcr": "", "overallExperience": "", "transfers": 0, "transfersCount": 0, "aht": 275, "talkTime": 268, "acw": 0, "holdTime": 6, "reliability": 0, "overallSentiment": 67.1, "positiveWord": 1.4, "negativeWord": 100, "managingEmotions": 100, "surveyTotal": 0, "totalCalls": 74}, {"name": "Alyssa Dimes", "firstName": "Alyssa", "scheduleAdherence": 88.67, "cxRepOverall": "", "fcr": "", "overallExperience": "", "transfers": 6.15, "transfersCount": 8, "aht": 678, "talkTime": 479, "acw": 64, "holdTime": 135, "reliability": 0, "overallSentiment": 94.7, "positiveWord": 96.9, "negativeWord": 90.1, "managingEmotions": 96.9, "surveyTotal": 0, "totalCalls": 130}, {"name": "Trisha Erb", "firstName": "Trisha", "scheduleAdherence": 90.06, "cxRepOverall": 100, "fcr": 0, "overallExperience": 100, "transfers": 7.04, "transfersCount": 5, "aht": 650, "talkTime": 412, "acw": 231, "holdTime": 7, "reliability": 0, "overallSentiment": 94.2, "positiveWord": 97.1, "negativeWord": 87, "managingEmotions": 98.6, "surveyTotal": 2, "totalCalls": 71}, {"name": "Angelina Fierro", "firstName": "Angelina", "scheduleAdherence": 83.46, "cxRepOverall": 100, "fcr": 100, "overallExperience": 100, "transfers": 3.67, "transfersCount": 4, "aht": 657, "talkTime": 486, "acw": 167, "holdTime": 4, "reliability": 0, "overallSentiment": 91.7, "positiveWord": 95.4, "negativeWord": 85.3, "managingEmotions": 94.5, "surveyTotal": 1, "totalCalls": 109}, {"name": "Jenifer Henson", "firstName": "Jenifer", "scheduleAdherence": 82.85, "cxRepOverall": 100, "fcr": 100, "overallExperience": 0, "transfers": 7.96, "transfersCount": 9, "aht": 535, "talkTime": 515, "acw": 0, "holdTime": 20, "reliability": 0, "overallSentiment": 89.6, "positiveWord": 93.8, "negativeWord": 83, "managingEmotions": 92, "surveyTotal": 1, "totalCalls": 113}, {"name": "Precious Johnson", "firstName": "Precious", "scheduleAdherence": 80.67, "cxRepOverall": 100, "fcr": 33.33, "overallExperience": 100, "transfers": 6.67, "transfersCount": 10, "aht": 392, "talkTime": 392, "acw": 0, "holdTime": 0, "reliability": 0, "overallSentiment": 93.8, "positiveWord": 99.3, "negativeWord": 84.1, "managingEmotions": 97.9, "surveyTotal": 3, "totalCalls": 150}, {"name": "Pamela Muhammad", "firstName": "Pamela", "scheduleAdherence": 95.42, "cxRepOverall": 50, "fcr": 0, "overallExperience": 50, "transfers": 32.82, "transfersCount": 86, "aht": 493, "talkTime": 392, "acw": 79, "holdTime": 22, "reliability": 0, "overallSentiment": 84.6, "positiveWord": 65.4, "negativeWord": 91.7, "managingEmotions": 96.9, "surveyTotal": 2, "totalCalls": 262}, {"name": "Scoticia Osborne", "firstName": "Scoticia", "scheduleAdherence": 90.78, "cxRepOverall": 100, "fcr": 100, "overallExperience": 100, "transfers": 7.69, "transfersCount": 14, "aht": 474, "talkTime": 433, "acw": 41, "holdTime": 0, "reliability": 0.3, "overallSentiment": 91.3, "positiveWord": 90, "negativeWord": 86.1, "managingEmotions": 97.8, "surveyTotal": 1, "totalCalls": 182}, {"name": "Trevor Pedrowski", "firstName": "Trevor", "scheduleAdherence": 86.16, "cxRepOverall": "", "fcr": "", "overallExperience": "", "transfers": 8.81, "transfersCount": 14, "aht": 467, "talkTime": 357, "acw": 89, "holdTime": 22, "reliability": 0, "overallSentiment": 79.3, "positiveWord": 66.4, "negativeWord": 79.3, "managingEmotions": 92.1, "surveyTotal": 0, "totalCalls": 159}, {"name": "Teena Pokorski", "firstName": "Teena", "scheduleAdherence": 94.71, "cxRepOverall": 100, "fcr": 100, "overallExperience": 100, "transfers": 8.26, "transfersCount": 18, "aht": 498, "talkTime": 368, "acw": 122, "holdTime": 8, "reliability": 0, "overallSentiment": 94.7, "positiveWord": 96.8, "negativeWord": 90.5, "managingEmotions": 96.8, "surveyTotal": 5, "totalCalls": 218}], "metadata": {"startDate": "2026-01-18", "endDate": "2026-01-24", "label": "Week ending Jan 24, 2026", "periodType": "week", "yearEndTargetProfile": "auto", "yearEndReviewYear": "2026", "uploadedAt": "2026-02-21T04:29:55.683Z"}}, "2026-01-25|2026-01-31": {"employees": [{"name": "Marietta Bernal", "firstName": "Marietta", "scheduleAdherence": 94.46, "cxRepOverall": 100, "fcr": 100, "overallExperience": 100, "transfers": 9.09, "transfersCount": 20, "aht": 378, "talkTime": 377, "acw": 0, "holdTime": 1, "reliability": 0, "overallSentiment": 87.6, "positiveWord": 78.9, "negativeWord": 87.6, "managingEmotions": 96.2, "surveyTotal": 4, "totalCalls": 220}, {"name": "Ekiecha Brabham", "firstName": "Ekiecha", "scheduleAdherence": 93.54, "cxRepOverall": 100, "fcr": 100, "overallExperience": 100, "transfers": 6.35, "transfersCount": 12, "aht": 512, "talkTime": 349, "acw": 129, "holdTime": 35, "reliability": 0, "overallSentiment": 86.4, "positiveWord": 84.2, "negativeWord": 81.9, "managingEmotions": 93.2, "surveyTotal": 1, "totalCalls": 189}, {"name": "Brittney Carroll", "firstName": "Brittney", "scheduleAdherence": 93.19, "cxRepOverall": 0, "fcr": 0, "overallExperience": 0, "transfers": 6.06, "transfersCount": 4, "aht": 733, "talkTime": 556, "acw": 160, "holdTime": 17, "reliability": 0, "overallSentiment": 90.6, "positiveWord": 96.9, "negativeWord": 79.7, "managingEmotions": 95.3, "surveyTotal": 1, "totalCalls": 66}, {"name": "Caylie Chirumbolo", "firstName": "Caylie", "scheduleAdherence": 86.7, "cxRepOverall": 100, "fcr": 100, "overallExperience": 50, "transfers": 4.14, "transfersCount": 7, "aht": 468, "talkTime": 332, "acw": 128, "holdTime": 8, "reliability": 0, "overallSentiment": 92.2, "positiveWord": 87.1, "negativeWord": 92.6, "managingEmotions": 96.9, "surveyTotal": 2, "totalCalls": 169}, {"name": "Darryn Coley", "firstName": "Darryn", "scheduleAdherence": 89.43, "cxRepOverall": "", "fcr": "", "overallExperience": "", "transfers": 17.5, "transfersCount": 35, "aht": 323, "talkTime": 202, "acw": 112, "holdTime": 9, "reliability": 11.78, "overallSentiment": 81, "positiveWord": 58.8, "negativeWord": 87.4, "managingEmotions": 96.7, "surveyTotal": 0, "totalCalls": 200}, {"name": "Ronda Colis", "firstName": "Ronda", "scheduleAdherence": 92.91, "cxRepOverall": 100, "fcr": 0, "overallExperience": 100, "transfers": 7.3, "transfersCount": 10, "aht": 824, "talkTime": 604, "acw": 211, "holdTime": 8, "reliability": 0, "overallSentiment": 91.2, "positiveWord": 95.5, "negativeWord": 83.5, "managingEmotions": 94.7, "surveyTotal": 1, "totalCalls": 137}, {"name": "Taylor Colter", "firstName": "Taylor", "scheduleAdherence": 99.36, "cxRepOverall": "", "fcr": "", "overallExperience": "", "transfers": 0, "transfersCount": 0, "aht": 237, "talkTime": 226, "acw": 0, "holdTime": 11, "reliability": 0, "overallSentiment": 66.7, "positiveWord": "", "negativeWord": 100, "managingEmotions": 100, "surveyTotal": 0, "totalCalls": 51}, {"name": "Alyssa Dimes", "firstName": "Alyssa", "scheduleAdherence": 96.11, "cxRepOverall": "", "fcr": "", "overallExperience": "", "transfers": 6.87, "transfersCount": 9, "aht": 518, "talkTime": 377, "acw": 28, "holdTime": 112, "reliability": 0, "overallSentiment": 95.9, "positiveWord": 96.9, "negativeWord": 91.5, "managingEmotions": 99.2, "surveyTotal": 0, "totalCalls": 131}, {"name": "Angelina Fierro", "firstName": "Angelina", "scheduleAdherence": 92.24, "cxRepOverall": 100, "fcr": 100, "overallExperience": 100, "transfers": 9.8, "transfersCount": 15, "aht": 732, "talkTime": 554, "acw": 176, "holdTime": 1, "reliability": 0, "overallSentiment": 94.3, "positiveWord": 98, "negativeWord": 89.5, "managingEmotions": 95.4, "surveyTotal": 1, "totalCalls": 153}, {"name": "Jenifer Henson", "firstName": "Jenifer", "scheduleAdherence": 93.74, "cxRepOverall": 100, "fcr": 100, "overallExperience": 100, "transfers": 11.4, "transfersCount": 22, "aht": 462, "talkTime": 444, "acw": 0, "holdTime": 18, "reliability": 0, "overallSentiment": 87.2, "positiveWord": 90.1, "negativeWord": 81.3, "managingEmotions": 90.1, "surveyTotal": 2, "totalCalls": 193}, {"name": "Precious Johnson", "firstName": "Precious", "scheduleAdherence": 85.63, "cxRepOverall": "", "fcr": "", "overallExperience": "", "transfers": 10.75, "transfersCount": 10, "aht": 408, "talkTime": 408, "acw": 0, "holdTime": 0, "reliability": 9.83, "overallSentiment": 92.2, "positiveWord": 98.9, "negativeWord": 82.2, "managingEmotions": 95.6, "surveyTotal": 0, "totalCalls": 93}, {"name": "Pamela Muhammad", "firstName": "Pamela", "scheduleAdherence": 92.7, "cxRepOverall": 100, "fcr": 100, "overallExperience": 100, "transfers": 26.09, "transfersCount": 48, "aht": 544, "talkTime": 446, "acw": 86, "holdTime": 13, "reliability": 0, "overallSentiment": 81.8, "positiveWord": 66.3, "negativeWord": 84, "managingEmotions": 95, "surveyTotal": 1, "totalCalls": 184}, {"name": "Scoticia Osborne", "firstName": "Scoticia", "scheduleAdherence": 92.08, "cxRepOverall": "", "fcr": "", "overallExperience": "", "transfers": 6.47, "transfersCount": 9, "aht": 424, "talkTime": 372, "acw": 52, "holdTime": 0, "reliability": 0, "overallSentiment": 93, "positiveWord": 97.8, "negativeWord": 84.9, "managingEmotions": 96.4, "surveyTotal": 0, "totalCalls": 139}, {"name": "Trevor Pedrowski", "firstName": "Trevor", "scheduleAdherence": 93.5, "cxRepOverall": 100, "fcr": 100, "overallExperience": 100, "transfers": 6.78, "transfersCount": 12, "aht": 542, "talkTime": 446, "acw": 69, "holdTime": 27, "reliability": 0, "overallSentiment": 84.6, "positiveWord": 73.4, "negativeWord": 85.5, "managingEmotions": 94.8, "surveyTotal": 1, "totalCalls": 177}, {"name": "Teena Pokorski", "firstName": "Teena", "scheduleAdherence": 95.05, "cxRepOverall": 100, "fcr": 100, "overallExperience": 100, "transfers": 8.07, "transfersCount": 13, "aht": 508, "talkTime": 382, "acw": 121, "holdTime": 5, "reliability": 0, "overallSentiment": 94.2, "positiveWord": 98.8, "negativeWord": 87.5, "managingEmotions": 96.3, "surveyTotal": 1, "totalCalls": 161}], "metadata": {"startDate": "2026-01-25", "endDate": "2026-01-31", "label": "Week ending Jan 31, 2026", "periodType": "week", "yearEndTargetProfile": "auto", "yearEndReviewYear": "2026", "uploadedAt": "2026-02-21T04:30:48.599Z"}}, "2026-02-01|2026-02-07": {"employees": [{"name": "Marietta Bernal", "firstName": "Marietta", "scheduleAdherence": 96.75, "cxRepOverall": 50, "fcr": 33.33, "overallExperience": 33.33, "transfers": 9.03, "transfersCount": 25, "aht": 343, "talkTime": 343, "acw": 0, "holdTime": 0, "reliability": 0, "overallSentiment": 85.4, "positiveWord": 72.9, "negativeWord": 90, "managingEmotions": 93.3, "surveyTotal": 3, "totalCalls": 277}, {"name": "Ekiecha Brabham", "firstName": "Ekiecha", "scheduleAdherence": 90.41, "cxRepOverall": "", "fcr": "", "overallExperience": "", "transfers": 9.09, "transfersCount": 17, "aht": 381, "talkTime": 260, "acw": 115, "holdTime": 6, "reliability": 6.25, "overallSentiment": 83.7, "positiveWord": 68.8, "negativeWord": 86.4, "managingEmotions": 96, "surveyTotal": 0, "totalCalls": 187}, {"name": "Brittney Carroll", "firstName": "Brittney", "scheduleAdherence": 94.93, "cxRepOverall": 100, "fcr": 100, "overallExperience": 100, "transfers": 4.08, "transfersCount": 4, "aht": 689, "talkTime": 476, "acw": 187, "holdTime": 26, "reliability": 0.5, "overallSentiment": 85.3, "positiveWord": 80, "negativeWord": 85.3, "managingEmotions": 90.5, "surveyTotal": 1, "totalCalls": 98}, {"name": "Caylie Chirumbolo", "firstName": "Caylie", "scheduleAdherence": 92.52, "cxRepOverall": 50, "fcr": 100, "overallExperience": 50, "transfers": 7.69, "transfersCount": 17, "aht": 409, "talkTime": 277, "acw": 124, "holdTime": 9, "reliability": 0.25, "overallSentiment": 92.9, "positiveWord": 89.4, "negativeWord": 93.1, "managingEmotions": 96.3, "surveyTotal": 2, "totalCalls": 221}, {"name": "Darryn Coley", "firstName": "Darryn", "scheduleAdherence": 92.24, "cxRepOverall": "", "fcr": "", "overallExperience": "", "transfers": 16.85, "transfersCount": 45, "aht": 300, "talkTime": 204, "acw": 76, "holdTime": 20, "reliability": 0, "overallSentiment": 78.4, "positiveWord": 50.4, "negativeWord": 89.8, "managingEmotions": 94.9, "surveyTotal": 0, "totalCalls": 267}, {"name": "Ronda Colis", "firstName": "Ronda", "scheduleAdherence": 88.24, "cxRepOverall": 100, "fcr": 100, "overallExperience": 100, "transfers": 4.17, "transfersCount": 4, "aht": 884, "talkTime": 660, "acw": 218, "holdTime": 6, "reliability": 2.5, "overallSentiment": 90.1, "positiveWord": 95.7, "negativeWord": 80.9, "managingEmotions": 93.6, "surveyTotal": 1, "totalCalls": 96}, {"name": "Taylor Colter", "firstName": "Taylor", "scheduleAdherence": 99.29, "cxRepOverall": "", "fcr": "", "overallExperience": "", "transfers": 0, "transfersCount": 0, "aht": 316, "talkTime": 313, "</t>
+          <t xml:space="preserve">{"generatedAt": "2026-02-25T19:58:06.007Z", "reason": "manual sync now", "sourceAppVersion": "2026.02.25.112", "weeklyData": {"2025-12-28|2026-01-03": {"employees": [{"name": "Marietta Bernal", "firstName": "Marietta", "scheduleAdherence": 97.67, "cxRepOverall": "", "fcr": "", "overallExperience": "", "transfers": 8.39, "transfersCount": 24, "aht": 404, "talkTime": 401, "acw": 0, "holdTime": 3, "reliability": 0, "overallSentiment": 83.2, "positiveWord": 77.3, "negativeWord": 78.4, "managingEmotions": 93.8, "surveyTotal": 0, "totalCalls": 286}, {"name": "Ekiecha Brabham", "firstName": "Ekiecha", "scheduleAdherence": 94.18, "cxRepOverall": "", "fcr": "", "overallExperience": "", "transfers": 6.94, "transfersCount": 12, "aht": 425, "talkTime": 251, "acw": 155, "holdTime": 18, "reliability": 0, "overallSentiment": 86.4, "positiveWord": 71.9, "negativeWord": 90.4, "managingEmotions": 97, "surveyTotal": 0, "totalCalls": 173}, {"name": "Caylie Chirumbolo", "firstName": "Caylie", "scheduleAdherence": 88.14, "cxRepOverall": 66.67, "fcr": 100, "overallExperience": 66.67, "transfers": 6.52, "transfersCount": 9, "aht": 468, "talkTime": 314, "acw": 128, "holdTime": 26, "reliability": 0.5, "overallSentiment": 92.8, "positiveWord": 90.3, "negativeWord": 91, "managingEmotions": 97, "surveyTotal": 3, "totalCalls": 138}, {"name": "Darryn Coley", "firstName": "Darryn", "scheduleAdherence": 89.41, "cxRepOverall": 0, "fcr": 100, "overallExperience": 0, "transfers": 8.84, "transfersCount": 16, "aht": 446, "talkTime": 248, "acw": 177, "holdTime": 21, "reliability": 0, "overallSentiment": 81.1, "positiveWord": 61.5, "negativeWord": 84.6, "managingEmotions": 97, "surveyTotal": 1, "totalCalls": 181}, {"name": "Ronda Colis", "firstName": "Ronda", "scheduleAdherence": 94.53, "cxRepOverall": "", "fcr": "", "overallExperience": "", "transfers": 5.68, "transfersCount": 5, "aht": 814, "talkTime": 591, "acw": 220, "holdTime": 3, "reliability": 0, "overallSentiment": 90.7, "positiveWord": 97.7, "negativeWord": 79.1, "managingEmotions": 95.3, "surveyTotal": 0, "totalCalls": 88}, {"name": "Taylor Colter", "firstName": "Taylor", "scheduleAdherence": 99.31, "cxRepOverall": "", "fcr": "", "overallExperience": "", "transfers": 0, "transfersCount": 0, "aht": 332, "talkTime": 315, "acw": 0, "holdTime": 17, "reliability": 0, "overallSentiment": 66.7, "positiveWord": "", "negativeWord": 100, "managingEmotions": 100, "surveyTotal": 0, "totalCalls": 72}, {"name": "Alyssa Dimes", "firstName": "Alyssa", "scheduleAdherence": 94.1, "cxRepOverall": "", "fcr": "", "overallExperience": "", "transfers": 5.1, "transfersCount": 8, "aht": 541, "talkTime": 378, "acw": 65, "holdTime": 98, "reliability": 0, "overallSentiment": 94.1, "positiveWord": 100, "negativeWord": 84.7, "managingEmotions": 97.5, "surveyTotal": 0, "totalCalls": 157}, {"name": "Trisha Erb", "firstName": "Trisha", "scheduleAdherence": 96.55, "cxRepOverall": "", "fcr": "", "overallExperience": "", "transfers": 10.43, "transfersCount": 12, "aht": 639, "talkTime": 466, "acw": 173, "holdTime": 0, "reliability": 0, "overallSentiment": 94.4, "positiveWord": 99.1, "negativeWord": 91.2, "managingEmotions": 92.9, "surveyTotal": 0, "totalCalls": 115}, {"name": "Angelina Fierro", "firstName": "Angelina", "scheduleAdherence": 93.43, "cxRepOverall": 100, "fcr": 100, "overallExperience": 100, "transfers": 6.72, "transfersCount": 9, "aht": 713, "talkTime": 545, "acw": 168, "holdTime": 0, "reliability": 0, "overallSentiment": 93.3, "positiveWord": 96.3, "negativeWord": 89.6, "managingEmotions": 94.1, "surveyTotal": 1, "totalCalls": 134}, {"name": "Jenifer Henson", "firstName": "Jenifer", "scheduleAdherence": 94, "cxRepOverall": "", "fcr": "", "overallExperience": "", "transfers": 7.65, "transfersCount": 13, "aht": 493, "talkTime": 478, "acw": 0, "holdTime": 15, "reliability": 0, "overallSentiment": 89.8, "positiveWord": 90.4, "negativeWord": 82.5, "managingEmotions": 96.4, "surveyTotal": 0, "totalCalls": 170}, {"name": "Oceane Ingram", "firstName": "Oceane", "scheduleAdherence": 86.78, "cxRepOverall": 100, "fcr": 100, "overallExperience": 100, "transfers": 12.31, "transfersCount": 16, "aht": 523, "talkTime": 271, "acw": 221, "holdTime": 32, "reliability": 0, "overallSentiment": 95.4, "positiveWord": 99.2, "negativeWord": 91.1, "managingEmotions": 95.9, "surveyTotal": 1, "totalCalls": 130}, {"name": "Precious Johnson", "firstName": "Precious", "scheduleAdherence": 93.88, "cxRepOverall": "", "fcr": "", "overallExperience": "", "transfers": 6.93, "transfersCount": 21, "aht": 371, "talkTime": 371, "acw": 1, "holdTime": 0, "reliability": 0, "overallSentiment": 93.4, "positiveWord": 97.7, "negativeWord": 85.7, "managingEmotions": 97, "surveyTotal": 0, "totalCalls": 303}, {"name": "Pamela Muhammad", "firstName": "Pamela", "scheduleAdherence": 94.43, "cxRepOverall": "", "fcr": "", "overallExperience": "", "transfers": 33.33, "transfersCount": 21, "aht": 782, "talkTime": 592, "acw": 171, "holdTime": 19, "reliability": 8.5, "overallSentiment": 85.7, "positiveWord": 73, "negativeWord": 87.3, "managingEmotions": 96.8, "surveyTotal": 0, "totalCalls": 63}, {"name": "Scoticia Osborne", "firstName": "Scoticia", "scheduleAdherence": 95.62, "cxRepOverall": "", "fcr": "", "overallExperience": "", "transfers": 3.85, "transfersCount": 5, "aht": 410, "talkTime": 364, "acw": 38, "holdTime": 8, "reliability": 0, "overallSentiment": 86.9, "positiveWord": 75.4, "negativeWord": 90, "managingEmotions": 95.4, "surveyTotal": 0, "totalCalls": 130}, {"name": "Teena Pokorski", "firstName": "Teena", "scheduleAdherence": 95.31, "cxRepOverall": 100, "fcr": 100, "overallExperience": 100, "transfers": 5.14, "transfersCount": 9, "aht": 514, "talkTime": 410, "acw": 98, "holdTime": 7, "reliability": 0, "overallSentiment": 94.3, "positiveWord": 98.3, "negativeWord": 88.5, "managingEmotions": 96, "surveyTotal": 2, "totalCalls": 175}], "metadata": {"startDate": "2025-12-28", "endDate": "2026-01-03", "label": "Week ending Jan 3, 2026", "periodType": "week", "yearEndTargetProfile": "auto", "yearEndReviewYear": "2026", "uploadedAt": "2026-02-21T04:27:22.786Z"}}, "2026-01-04|2026-01-10": {"employees": [{"name": "Ekiecha Brabham", "firstName": "Ekiecha", "scheduleAdherence": 89.85, "cxRepOverall": "", "fcr": "", "overallExperience": "", "transfers": 6.4, "transfersCount": 8, "aht": 455, "talkTime": 295, "acw": 150, "holdTime": 10, "reliability": 0, "overallSentiment": 81.6, "positiveWord": 69.5, "negativeWord": 80.5, "managingEmotions": 94.9, "surveyTotal": 0, "totalCalls": 125}, {"name": "Caylie Chirumbolo", "firstName": "Caylie", "scheduleAdherence": 84.5, "cxRepOverall": 0, "fcr": 0, "overallExperience": 0, "transfers": 9.78, "transfersCount": 18, "aht": 475, "talkTime": 321, "acw": 145, "holdTime": 10, "reliability": 0, "overallSentiment": 90.3, "positiveWord": 88.3, "negativeWord": 88.8, "managingEmotions": 93.9, "surveyTotal": 1, "totalCalls": 184}, {"name": "Darryn Coley", "firstName": "Darryn", "scheduleAdherence": 89.97, "cxRepOverall": "", "fcr": "", "overallExperience": "", "transfers": 11.21, "transfersCount": 13, "aht": 500, "talkTime": 355, "acw": 130, "holdTime": 16, "reliability": 0, "overallSentiment": 80.4, "positiveWord": 66.3, "negativeWord": 79.8, "managingEmotions": 95.2, "surveyTotal": 0, "totalCalls": 116}, {"name": "Ronda Colis", "firstName": "Ronda", "scheduleAdherence": 92.62, "cxRepOverall": "", "fcr": "", "overallExperience": "", "transfers": 4.49, "transfersCount": 4, "aht": 878, "talkTime": 651, "acw": 224, "holdTime": 2, "reliability": 0, "overallSentiment": 88.5, "positiveWord": 93.1, "negativeWord": 81.6, "managingEmotions": 90.8, "surveyTotal": 0, "totalCalls": 89}, {"name": "Taylor Colter", "firstName": "Taylor", "scheduleAdherence": 98.79, "cxRepOverall": "", "fcr": "", "overallExperience": "", "transfers": 0, "transfersCount": 0, "aht": 256, "talkTime": 248, "acw": 0, "holdTime": 7, "reliability": 0, "overallSentiment": 67.2, "positiveWord": 1.5, "negativeWord": 100, "managingEmotions": 100, "surveyTotal": 0, "totalCalls": 75}, {"name": "Alyssa Dimes", "firstName": "Alyssa", "scheduleAdherence": 94.28, "cxRepOverall": "", "fcr": "", "overallExperience": "", "transfers": 5.32, "transfersCount": 5, "aht": 628, "talkTime": 455, "acw": 69, "holdTime": 104, "reliability": 0, "overallSentiment": 92.2, "positiveWord": 97.9, "negativeWord": 85.1, "managingEmotions": 93.6, "surveyTotal": 0, "totalCalls": 94}, {"name": "Trisha Erb", "firstName": "Trisha", "scheduleAdherence": 95.22, "cxRepOverall": 100, "fcr": 100, "overallExperience": 100, "transfers": 10.18, "transfersCount": 17, "aht": 693, "talkTime": 479, "acw": 211, "holdTime": 3, "reliability": 0, "overallSentiment": 91.8, "positiveWord": 97, "negativeWord": 86.8, "managingEmotions": 91.6, "surveyTotal": 1, "totalCalls": 167}, {"name": "Angelina Fierro", "firstName": "Angelina", "scheduleAdherence": 90.95, "cxRepOverall": 100, "fcr": 100, "overallExperience": 100, "transfers": 12, "transfersCount": 18, "aht": 737, "talkTime": 562, "acw": 173, "holdTime": 2, "reliability": 0, "overallSentiment": 93.3, "positiveWord": 98, "negativeWord": 86, "managingEmotions": 96, "surveyTotal": 2, "totalCalls": 150}, {"name": "Jenifer Henson", "firstName": "Jenifer", "scheduleAdherence": 94.74, "cxRepOverall": 100, "fcr": 100, "overallExperience": 100, "transfers": 13.02, "transfersCount": 22, "aht": 491, "talkTime": 477, "acw": 0, "holdTime": 14, "reliability": 0, "overallSentiment": 87.8, "positiveWord": 89.2, "negativeWord": 77.8, "managingEmotions": 96.4, "surveyTotal": 1, "totalCalls": 169}, {"name": "Oceane Ingram", "firstName": "Oceane", "scheduleAdherence": 84.27, "cxRepOverall": 100, "fcr": 0, "overallExperience": 100, "transfers": 11.49, "transfersCount": 17, "aht": 551, "talkTime": 259, "acw": 246, "holdTime": 46, "reliability": 0, "overallSentiment": 95.6, "positiveWord": 98.6, "negativeWord": 93.7, "managingEmotions": 94.4, "surveyTotal": 1, "totalCalls": 148}, {"name": "Precious Johnson", "firstName": "Precious", "scheduleAdherence": 91.87, "cxRepOverall": 100, "fcr": 100, "overallExperience": 100, "transfers": 6.11, "transfersCount": 11, "aht": 430, "talkTime": 430, "acw": 0, "holdTime": 0, "reliability": 0, "overallSentiment": 94, "positiveWord": 99.4, "negativeWord": 87.2, "managingEmotions": 95.5, "surveyTotal": 3, "totalCalls": 180}, {"name": "Pamela Muhammad", "firstName": "Pamela", "scheduleAdherence": 98.66, "cxRepOverall": "", "fcr": "", "overallExperience": "", "transfers": 23.73, "transfersCount": 28, "aht": 694, "talkTime": 561, "acw": 93, "holdTime": 40, "reliability": 0, "overallSentiment": 90.5, "positiveWord": 84.5, "negativeWord": 90.5, "managingEmotions": 96.6, "surveyTotal": 0, "totalCalls": 118}, {"name": "Scoticia Osborne", "firstName": "Scoticia", "scheduleAdherence": 91.66, "cxRepOverall": 100, "fcr": 50, "overallExperience": 100, "transfers": 5, "transfersCount": 5, "aht": 451, "talkTime": 410, "acw": 38, "holdTime": 3, "reliability": 0, "overallSentiment": 89.1, "positiveWord": 90.5, "negativeWord": 83.2, "managingEmotions": 93.7, "surveyTotal": 2, "totalCalls": 100}, {"name": "Trevor Pedrowski", "firstName": "Trevor", "scheduleAdherence": 90.5, "cxRepOverall": 100, "fcr": "", "overallExperience": "", "transfers": 7.14, "transfersCount": 11, "aht": 470, "talkTime": 368, "acw": 91, "holdTime": 10, "reliability": 0, "overallSentiment": 84.1, "positiveWord": 75.5, "negativeWord": 81.6, "managingEmotions": 95.2, "surveyTotal": 0, "totalCalls": 154}, {"name": "Teena Pokorski", "firstName": "Teena", "scheduleAdherence": 92.96, "cxRepOverall": 100, "fcr": 50, "overallExperience": 100, "transfers": 7.94, "transfersCount": 17, "aht": 506, "talkTime": 387, "acw": 111, "holdTime": 8, "reliability": 0, "overallSentiment": 94.3, "positiveWord": 95.9, "negativeWord": 90.4, "managingEmotions": 96.8, "surveyTotal": 2, "totalCalls": 214}], "metadata": {"startDate": "2026-01-04", "endDate": "2026-01-10", "label": "Week ending Jan 10, 2026", "periodType": "week", "yearEndTargetProfile": "auto", "yearEndReviewYear": "2026", "uploadedAt": "2026-02-21T04:28:01.178Z"}}, "2026-01-11|2026-01-17": {"employees": [{"name": "Marietta Bernal", "firstName": "Marietta", "scheduleAdherence": 94.58, "cxRepOverall": 75, "fcr": 50, "overallExperience": 50, "transfers": 13.06, "transfersCount": 32, "aht": 434, "talkTime": 434, "acw": 0, "holdTime": 1, "reliability": 0, "overallSentiment": 80.5, "positiveWord": 70.2, "negativeWord": 76.9, "managingEmotions": 94.5, "surveyTotal": 4, "totalCalls": 245}, {"name": "Ekiecha Brabham", "firstName": "Ekiecha", "scheduleAdherence": 89.63, "cxRepOverall": 100, "fcr": 33.33, "overallExperience": 100, "transfers": 7.69, "transfersCount": 10, "aht": 417, "talkTime": 242, "acw": 146, "holdTime": 29, "reliability": 0, "overallSentiment": 85, "positiveWord": 68.3, "negativeWord": 89.2, "managingEmotions": 97.5, "surveyTotal": 3, "totalCalls": 130}, {"name": "Caylie Chirumbolo", "firstName": "Caylie", "scheduleAdherence": 91.44, "cxRepOverall": "", "fcr": "", "overallExperience": "", "transfers": 4.81, "transfersCount": 10, "aht": 460, "talkTime": 320, "acw": 124, "holdTime": 16, "reliability": 0.3, "overallSentiment": 92.6, "positiveWord": 94, "negativeWord": 85.4, "managingEmotions": 98.5, "surveyTotal": 0, "totalCalls": 208}, {"name": "Darryn Coley", "firstName": "Darryn", "scheduleAdherence": 80.17, "cxRepOverall": "", "fcr": "", "overallExperience": "", "transfers": 11.66, "transfersCount": 19, "aht": 517, "talkTime": 282, "acw": 201, "holdTime": 35, "reliability": 0.28, "overallSentiment": 83.3, "positiveWord": 72.3, "negativeWord": 82.4, "managingEmotions": 95.3, "surveyTotal": 0, "totalCalls": 163}, {"name": "Ronda Colis", "firstName": "Ronda", "scheduleAdherence": 93.85, "cxRepOverall": 100, "fcr": 100, "overallExperience": 50, "transfers": 5.15, "transfersCount": 5, "aht": 883, "talkTime": 650, "acw": 231, "holdTime": 2, "reliability": 0, "overallSentiment": 89.9, "positiveWord": 90.6, "negativeWord": 83.3, "managingEmotions": 95.8, "surveyTotal": 2, "totalCalls": 97}, {"name": "Taylor Colter", "firstName": "Taylor", "scheduleAdherence": 97.43, "cxRepOverall": "", "fcr": "", "overallExperience": "", "transfers": 0, "transfersCount": 0, "aht": 275, "talkTime": 268, "acw": 0, "holdTime": 6, "reliability": 0, "overallSentiment": 67.1, "positiveWord": 1.4, "negativeWord": 100, "managingEmotions": 100, "surveyTotal": 0, "totalCalls": 74}, {"name": "Alyssa Dimes", "firstName": "Alyssa", "scheduleAdherence": 88.67, "cxRepOverall": "", "fcr": "", "overallExperience": "", "transfers": 6.15, "transfersCount": 8, "aht": 678, "talkTime": 479, "acw": 64, "holdTime": 135, "reliability": 0, "overallSentiment": 94.7, "positiveWord": 96.9, "negativeWord": 90.1, "managingEmotions": 96.9, "surveyTotal": 0, "totalCalls": 130}, {"name": "Trisha Erb", "firstName": "Trisha", "scheduleAdherence": 90.06, "cxRepOverall": 100, "fcr": 0, "overallExperience": 100, "transfers": 7.04, "transfersCount": 5, "aht": 650, "talkTime": 412, "acw": 231, "holdTime": 7, "reliability": 0, "overallSentiment": 94.2, "positiveWord": 97.1, "negativeWord": 87, "managingEmotions": 98.6, "surveyTotal": 2, "totalCalls": 71}, {"name": "Angelina Fierro", "firstName": "Angelina", "scheduleAdherence": 83.46, "cxRepOverall": 100, "fcr": 100, "overallExperience": 100, "transfers": 3.67, "transfersCount": 4, "aht": 657, "talkTime": 486, "acw": 167, "holdTime": 4, "reliability": 0, "overallSentiment": 91.7, "positiveWord": 95.4, "negativeWord": 85.3, "managingEmotions": 94.5, "surveyTotal": 1, "totalCalls": 109}, {"name": "Jenifer Henson", "firstName": "Jenifer", "scheduleAdherence": 82.85, "cxRepOverall": 100, "fcr": 100, "overallExperience": 0, "transfers": 7.96, "transfersCount": 9, "aht": 535, "talkTime": 515, "acw": 0, "holdTime": 20, "reliability": 0, "overallSentiment": 89.6, "positiveWord": 93.8, "negativeWord": 83, "managingEmotions": 92, "surveyTotal": 1, "totalCalls": 113}, {"name": "Precious Johnson", "firstName": "Precious", "scheduleAdherence": 80.67, "cxRepOverall": 100, "fcr": 33.33, "overallExperience": 100, "transfers": 6.67, "transfersCount": 10, "aht": 392, "talkTime": 392, "acw": 0, "holdTime": 0, "reliability": 0, "overallSentiment": 93.8, "positiveWord": 99.3, "negativeWord": 84.1, "managingEmotions": 97.9, "surveyTotal": 3, "totalCalls": 150}, {"name": "Pamela Muhammad", "firstName": "Pamela", "scheduleAdherence": 95.42, "cxRepOverall": 50, "fcr": 0, "overallExperience": 50, "transfers": 32.82, "transfersCount": 86, "aht": 493, "talkTime": 392, "acw": 79, "holdTime": 22, "reliability": 0, "overallSentiment": 84.6, "positiveWord": 65.4, "negativeWord": 91.7, "managingEmotions": 96.9, "surveyTotal": 2, "totalCalls": 262}, {"name": "Scoticia Osborne", "firstName": "Scoticia", "scheduleAdherence": 90.78, "cxRepOverall": 100, "fcr": 100, "overallExperience": 100, "transfers": 7.69, "transfersCount": 14, "aht": 474, "talkTime": 433, "acw": 41, "holdTime": 0, "reliability": 0.3, "overallSentiment": 91.3, "positiveWord": 90, "negativeWord": 86.1, "managingEmotions": 97.8, "surveyTotal": 1, "totalCalls": 182}, {"name": "Trevor Pedrowski", "firstName": "Trevor", "scheduleAdherence": 86.16, "cxRepOverall": "", "fcr": "", "overallExperience": "", "transfers": 8.81, "transfersCount": 14, "aht": 467, "talkTime": 357, "acw": 89, "holdTime": 22, "reliability": 0, "overallSentiment": 79.3, "positiveWord": 66.4, "negativeWord": 79.3, "managingEmotions": 92.1, "surveyTotal": 0, "totalCalls": 159}, {"name": "Teena Pokorski", "firstName": "Teena", "scheduleAdherence": 94.71, "cxRepOverall": 100, "fcr": 100, "overallExperience": 100, "transfers": 8.26, "transfersCount": 18, "aht": 498, "talkTime": 368, "acw": 122, "holdTime": 8, "reliability": 0, "overallSentiment": 94.7, "positiveWord": 96.8, "negativeWord": 90.5, "managingEmotions": 96.8, "surveyTotal": 5, "totalCalls": 218}], "metadata": {"startDate": "2026-01-11", "endDate": "2026-01-17", "label": "Week ending Jan 17, 2026", "periodType": "week", "yearEndTargetProfile": "auto", "yearEndReviewYear": "2026", "uploadedAt": "2026-02-21T04:29:28.383Z"}}, "2026-01-18|2026-01-24": {"employees": [{"name": "Marietta Bernal", "firstName": "Marietta", "scheduleAdherence": 94.58, "cxRepOverall": 75, "fcr": 50, "overallExperience": 50, "transfers": 13.06, "transfersCount": 32, "aht": 434, "talkTime": 434, "acw": 0, "holdTime": 1, "reliability": 0, "overallSentiment": 80.5, "positiveWord": 70.2, "negativeWord": 76.9, "managingEmotions": 94.5, "surveyTotal": 4, "totalCalls": 245}, {"name": "Ekiecha Brabham", "firstName": "Ekiecha", "scheduleAdherence": 89.63, "cxRepOverall": 100, "fcr": 33.33, "overallExperience": 100, "transfers": 7.69, "transfersCount": 10, "aht": 417, "talkTime": 242, "acw": 146, "holdTime": 29, "reliability": 0, "overallSentiment": 85, "positiveWord": 68.3, "negativeWord": 89.2, "managingEmotions": 97.5, "surveyTotal": 3, "totalCalls": 130}, {"name": "Caylie Chirumbolo", "firstName": "Caylie", "scheduleAdherence": 91.44, "cxRepOverall": "", "fcr": "", "overallExperience": "", "transfers": 4.81, "transfersCount": 10, "aht": 460, "talkTime": 320, "acw": 124, "holdTime": 16, "reliability": 0.3, "overallSentiment": 92.6, "positiveWord": 94, "negativeWord": 85.4, "managingEmotions": 98.5, "surveyTotal": 0, "totalCalls": 208}, {"name": "Darryn Coley", "firstName": "Darryn", "scheduleAdherence": 80.17, "cxRepOverall": "", "fcr": "", "overallExperience": "", "transfers": 11.66, "transfersCount": 19, "aht": 517, "talkTime": 282, "acw": 201, "holdTime": 35, "reliability": 0.28, "overallSentiment": 83.3, "positiveWord": 72.3, "negativeWord": 82.4, "managingEmotions": 95.3, "surveyTotal": 0, "totalCalls": 163}, {"name": "Ronda Colis", "firstName": "Ronda", "scheduleAdherence": 93.85, "cxRepOverall": 100, "fcr": 100, "overallExperience": 50, "transfers": 5.15, "transfersCount": 5, "aht": 883, "talkTime": 650, "acw": 231, "holdTime": 2, "reliability": 0, "overallSentiment": 89.9, "positiveWord": 90.6, "negativeWord": 83.3, "managingEmotions": 95.8, "surveyTotal": 2, "totalCalls": 97}, {"name": "Taylor Colter", "firstName": "Taylor", "scheduleAdherence": 97.43, "cxRepOverall": "", "fcr": "", "overallExperience": "", "transfers": 0, "transfersCount": 0, "aht": 275, "talkTime": 268, "acw": 0, "holdTime": 6, "reliability": 0, "overallSentiment": 67.1, "positiveWord": 1.4, "negativeWord": 100, "managingEmotions": 100, "surveyTotal": 0, "totalCalls": 74}, {"name": "Alyssa Dimes", "firstName": "Alyssa", "scheduleAdherence": 88.67, "cxRepOverall": "", "fcr": "", "overallExperience": "", "transfers": 6.15, "transfersCount": 8, "aht": 678, "talkTime": 479, "acw": 64, "holdTime": 135, "reliability": 0, "overallSentiment": 94.7, "positiveWord": 96.9, "negativeWord": 90.1, "managingEmotions": 96.9, "surveyTotal": 0, "totalCalls": 130}, {"name": "Trisha Erb", "firstName": "Trisha", "scheduleAdherence": 90.06, "cxRepOverall": 100, "fcr": 0, "overallExperience": 100, "transfers": 7.04, "transfersCount": 5, "aht": 650, "talkTime": 412, "acw": 231, "holdTime": 7, "reliability": 0, "overallSentiment": 94.2, "positiveWord": 97.1, "negativeWord": 87, "managingEmotions": 98.6, "surveyTotal": 2, "totalCalls": 71}, {"name": "Angelina Fierro", "firstName": "Angelina", "scheduleAdherence": 83.46, "cxRepOverall": 100, "fcr": 100, "overallExperience": 100, "transfers": 3.67, "transfersCount": 4, "aht": 657, "talkTime": 486, "acw": 167, "holdTime": 4, "reliability": 0, "overallSentiment": 91.7, "positiveWord": 95.4, "negativeWord": 85.3, "managingEmotions": 94.5, "surveyTotal": 1, "totalCalls": 109}, {"name": "Jenifer Henson", "firstName": "Jenifer", "scheduleAdherence": 82.85, "cxRepOverall": 100, "fcr": 100, "overallExperience": 0, "transfers": 7.96, "transfersCount": 9, "aht": 535, "talkTime": 515, "acw": 0, "holdTime": 20, "reliability": 0, "overallSentiment": 89.6, "positiveWord": 93.8, "negativeWord": 83, "managingEmotions": 92, "surveyTotal": 1, "totalCalls": 113}, {"name": "Precious Johnson", "firstName": "Precious", "scheduleAdherence": 80.67, "cxRepOverall": 100, "fcr": 33.33, "overallExperience": 100, "transfers": 6.67, "transfersCount": 10, "aht": 392, "talkTime": 392, "acw": 0, "holdTime": 0, "reliability": 0, "overallSentiment": 93.8, "positiveWord": 99.3, "negativeWord": 84.1, "managingEmotions": 97.9, "surveyTotal": 3, "totalCalls": 150}, {"name": "Pamela Muhammad", "firstName": "Pamela", "scheduleAdherence": 95.42, "cxRepOverall": 50, "fcr": 0, "overallExperience": 50, "transfers": 32.82, "transfersCount": 86, "aht": 493, "talkTime": 392, "acw": 79, "holdTime": 22, "reliability": 0, "overallSentiment": 84.6, "positiveWord": 65.4, "negativeWord": 91.7, "managingEmotions": 96.9, "surveyTotal": 2, "totalCalls": 262}, {"name": "Scoticia Osborne", "firstName": "Scoticia", "scheduleAdherence": 90.78, "cxRepOverall": 100, "fcr": 100, "overallExperience": 100, "transfers": 7.69, "transfersCount": 14, "aht": 474, "talkTime": 433, "acw": 41, "holdTime": 0, "reliability": 0.3, "overallSentiment": 91.3, "positiveWord": 90, "negativeWord": 86.1, "managingEmotions": 97.8, "surveyTotal": 1, "totalCalls": 182}, {"name": "Trevor Pedrowski", "firstName": "Trevor", "scheduleAdherence": 86.16, "cxRepOverall": "", "fcr": "", "overallExperience": "", "transfers": 8.81, "transfersCount": 14, "aht": 467, "talkTime": 357, "acw": 89, "holdTime": 22, "reliability": 0, "overallSentiment": 79.3, "positiveWord": 66.4, "negativeWord": 79.3, "managingEmotions": 92.1, "surveyTotal": 0, "totalCalls": 159}, {"name": "Teena Pokorski", "firstName": "Teena", "scheduleAdherence": 94.71, "cxRepOverall": 100, "fcr": 100, "overallExperience": 100, "transfers": 8.26, "transfersCount": 18, "aht": 498, "talkTime": 368, "acw": 122, "holdTime": 8, "reliability": 0, "overallSentiment": 94.7, "positiveWord": 96.8, "negativeWord": 90.5, "managingEmotions": 96.8, "surveyTotal": 5, "totalCalls": 218}], "metadata": {"startDate": "2026-01-18", "endDate": "2026-01-24", "label": "Week ending Jan 24, 2026", "periodType": "week", "yearEndTargetProfile": "auto", "yearEndReviewYear": "2026", "uploadedAt": "2026-02-21T04:29:55.683Z"}}, "2026-01-25|2026-01-31": {"employees": [{"name": "Marietta Bernal", "firstName": "Marietta", "scheduleAdherence": 94.46, "cxRepOverall": 100, "fcr": 100, "overallExperience": 100, "transfers": 9.09, "transfersCount": 20, "aht": 378, "talkTime": 377, "acw": 0, "holdTime": 1, "reliability": 0, "overallSentiment": 87.6, "positiveWord": 78.9, "negativeWord": 87.6, "managingEmotions": 96.2, "surveyTotal": 4, "totalCalls": 220}, {"name": "Ekiecha Brabham", "firstName": "Ekiecha", "scheduleAdherence": 93.54, "cxRepOverall": 100, "fcr": 100, "overallExperience": 100, "transfers": 6.35, "transfersCount": 12, "aht": 512, "talkTime": 349, "acw": 129, "holdTime": 35, "reliability": 0, "overallSentiment": 86.4, "positiveWord": 84.2, "negativeWord": 81.9, "managingEmotions": 93.2, "surveyTotal": 1, "totalCalls": 189}, {"name": "Brittney Carroll", "firstName": "Brittney", "scheduleAdherence": 93.19, "cxRepOverall": 0, "fcr": 0, "overallExperience": 0, "transfers": 6.06, "transfersCount": 4, "aht": 733, "talkTime": 556, "acw": 160, "holdTime": 17, "reliability": 0, "overallSentiment": 90.6, "positiveWord": 96.9, "negativeWord": 79.7, "managingEmotions": 95.3, "surveyTotal": 1, "totalCalls": 66}, {"name": "Caylie Chirumbolo", "firstName": "Caylie", "scheduleAdherence": 86.7, "cxRepOverall": 100, "fcr": 100, "overallExperience": 50, "transfers": 4.14, "transfersCount": 7, "aht": 468, "talkTime": 332, "acw": 128, "holdTime": 8, "reliability": 0, "overallSentiment": 92.2, "positiveWord": 87.1, "negativeWord": 92.6, "managingEmotions": 96.9, "surveyTotal": 2, "totalCalls": 169}, {"name": "Darryn Coley", "firstName": "Darryn", "scheduleAdherence": 89.43, "cxRepOverall": "", "fcr": "", "overallExperience": "", "transfers": 17.5, "transfersCount": 35, "aht": 323, "talkTime": 202, "acw": 112, "holdTime": 9, "reliability": 11.78, "overallSentiment": 81, "positiveWord": 58.8, "negativeWord": 87.4, "managingEmotions": 96.7, "surveyTotal": 0, "totalCalls": 200}, {"name": "Ronda Colis", "firstName": "Ronda", "scheduleAdherence": 92.91, "cxRepOverall": 100, "fcr": 0, "overallExperience": 100, "transfers": 7.3, "transfersCount": 10, "aht": 824, "talkTime": 604, "acw": 211, "holdTime": 8, "reliability": 0, "overallSentiment": 91.2, "positiveWord": 95.5, "negativeWord": 83.5, "managingEmotions": 94.7, "surveyTotal": 1, "totalCalls": 137}, {"name": "Taylor Colter", "firstName": "Taylor", "scheduleAdherence": 99.36, "cxRepOverall": "", "fcr": "", "overallExperience": "", "transfers": 0, "transfersCount": 0, "aht": 237, "talkTime": 226, "acw": 0, "holdTime": 11, "reliability": 0, "overallSentiment": 66.7, "positiveWord": "", "negativeWord": 100, "managingEmotions": 100, "surveyTotal": 0, "totalCalls": 51}, {"name": "Alyssa Dimes", "firstName": "Alyssa", "scheduleAdherence": 96.11, "cxRepOverall": "", "fcr": "", "overallExperience": "", "transfers": 6.87, "transfersCount": 9, "aht": 518, "talkTime": 377, "acw": 28, "holdTime": 112, "reliability": 0, "overallSentiment": 95.9, "positiveWord": 96.9, "negativeWord": 91.5, "managingEmotions": 99.2, "surveyTotal": 0, "totalCalls": 131}, {"name": "Angelina Fierro", "firstName": "Angelina", "scheduleAdherence": 92.24, "cxRepOverall": 100, "fcr": 100, "overallExperience": 100, "transfers": 9.8, "transfersCount": 15, "aht": 732, "talkTime": 554, "acw": 176, "holdTime": 1, "reliability": 0, "overallSentiment": 94.3, "positiveWord": 98, "negativeWord": 89.5, "managingEmotions": 95.4, "surveyTotal": 1, "totalCalls": 153}, {"name": "Jenifer Henson", "firstName": "Jenifer", "scheduleAdherence": 93.74, "cxRepOverall": 100, "fcr": 100, "overallExperience": 100, "transfers": 11.4, "transfersCount": 22, "aht": 462, "talkTime": 444, "acw": 0, "holdTime": 18, "reliability": 0, "overallSentiment": 87.2, "positiveWord": 90.1, "negativeWord": 81.3, "managingEmotions": 90.1, "surveyTotal": 2, "totalCalls": 193}, {"name": "Precious Johnson", "firstName": "Precious", "scheduleAdherence": 85.63, "cxRepOverall": "", "fcr": "", "overallExperience": "", "transfers": 10.75, "transfersCount": 10, "aht": 408, "talkTime": 408, "acw": 0, "holdTime": 0, "reliability": 9.83, "overallSentiment": 92.2, "positiveWord": 98.9, "negativeWord": 82.2, "managingEmotions": 95.6, "surveyTotal": 0, "totalCalls": 93}, {"name": "Pamela Muhammad", "firstName": "Pamela", "scheduleAdherence": 92.7, "cxRepOverall": 100, "fcr": 100, "overallExperience": 100, "transfers": 26.09, "transfersCount": 48, "aht": 544, "talkTime": 446, "acw": 86, "holdTime": 13, "reliability": 0, "overallSentiment": 81.8, "positiveWord": 66.3, "negativeWord": 84, "managingEmotions": 95, "surveyTotal": 1, "totalCalls": 184}, {"name": "Scoticia Osborne", "firstName": "Scoticia", "scheduleAdherence": 92.08, "cxRepOverall": "", "fcr": "", "overallExperience": "", "transfers": 6.47, "transfersCount": 9, "aht": 424, "talkTime": 372, "acw": 52, "holdTime": 0, "reliability": 0, "overallSentiment": 93, "positiveWord": 97.8, "negativeWord": 84.9, "managingEmotions": 96.4, "surveyTotal": 0, "totalCalls": 139}, {"name": "Trevor Pedrowski", "firstName": "Trevor", "scheduleAdherence": 93.5, "cxRepOverall": 100, "fcr": 100, "overallExperience": 100, "transfers": 6.78, "transfersCount": 12, "aht": 542, "talkTime": 446, "acw": 69, "holdTime": 27, "reliability": 0, "overallSentiment": 84.6, "positiveWord": 73.4, "negativeWord": 85.5, "managingEmotions": 94.8, "surveyTotal": 1, "totalCalls": 177}, {"name": "Teena Pokorski", "firstName": "Teena", "scheduleAdherence": 95.05, "cxRepOverall": 100, "fcr": 100, "overallExperience": 100, "transfers": 8.07, "transfersCount": 13, "aht": 508, "talkTime": 382, "acw": 121, "holdTime": 5, "reliability": 0, "overallSentiment": 94.2, "positiveWord": 98.8, "negativeWord": 87.5, "managingEmotions": 96.3, "surveyTotal": 1, "totalCalls": 161}], "metadata": {"startDate": "2026-01-25", "endDate": "2026-01-31", "label": "Week ending Jan 31, 2026", "periodType": "week", "yearEndTargetProfile": "auto", "yearEndReviewYear": "2026", "uploadedAt": "2026-02-21T04:30:48.599Z"}}, "2026-02-01|2026-02-07": {"employees": [{"name": "Marietta Bernal", "firstName": "Marietta", "scheduleAdherence": 96.75, "cxRepOverall": 50, "fcr": 33.33, "overallExperience": 33.33, "transfers": 9.03, "transfersCount": 25, "aht": 343, "talkTime": 343, "acw": 0, "holdTime": 0, "reliability": 0, "overallSentiment": 85.4, "positiveWord": 72.9, "negativeWord": 90, "managingEmotions": 93.3, "surveyTotal": 3, "totalCalls": 277}, {"name": "Ekiecha Brabham", "firstName": "Ekiecha", "scheduleAdherence": 90.41, "cxRepOverall": "", "fcr": "", "overallExperience": "", "transfers": 9.09, "transfersCount": 17, "aht": 381, "talkTime": 260, "acw": 115, "holdTime": 6, "reliability": 6.25, "overallSentiment": 83.7, "positiveWord": 68.8, "negativeWord": 86.4, "managingEmotions": 96, "surveyTotal": 0, "totalCalls": 187}, {"name": "Brittney Carroll", "firstName": "Brittney", "scheduleAdherence": 94.93, "cxRepOverall": 100, "fcr": 100, "overallExperience": 100, "transfers": 4.08, "transfersCount": 4, "aht": 689, "talkTime": 476, "acw": 187, "holdTime": 26, "reliability": 0.5, "overallSentiment": 85.3, "positiveWord": 80, "negativeWord": 85.3, "managingEmotions": 90.5, "surveyTotal": 1, "totalCalls": 98}, {"name": "Caylie Chirumbolo", "firstName": "Caylie", "scheduleAdherence": 92.52, "cxRepOverall": 50, "fcr": 100, "overallExperience": 50, "transfers": 7.69, "transfersCount": 17, "aht": 409, "talkTime": 277, "acw": 124, "holdTime": 9, "reliability": 0.25, "overallSentiment": 92.9, "positiveWord": 89.4, "negativeWord": 93.1, "managingEmotions": 96.3, "surveyTotal": 2, "totalCalls": 221}, {"name": "Darryn Coley", "firstName": "Darryn", "scheduleAdherence": 92.24, "cxRepOverall": "", "fcr": "", "overallExperience": "", "transfers": 16.85, "transfersCount": 45, "aht": 300, "talkTime": 204, "acw": 76, "holdTime": 20, "reliability": 0, "overallSentiment": 78.4, "positiveWord": 50.4, "negativeWord": 89.8, "managingEmotions": 94.9, "surveyTotal": 0, "totalCalls": 267}, {"name": "Ronda Colis", "firstName": "Ronda", "scheduleAdherence": 88.24, "cxRepOverall": 100, "fcr": 100, "overallExperience": 100, "transfers": 4.17, "transfersCount": 4, "aht": 884, "talkTime": 660, "acw": 218, "holdTime": 6, "reliability": 2.5, "overallSentiment": 90.1, "positiveWord": 95.7, "negativeWord": 80.9, "managingEmotions": 93.6, "surveyTotal": 1, "totalCalls": 96}, {"name": "Taylor Colter", "firstName": "Taylor", "scheduleAdherence": 99.29, "cxRepOverall": "", "fcr": "", "overallExperience": "", "transfers": 0, "transfersCount": 0, "aht": 316, "talkTime": 313, </t>
         </is>
       </c>
     </row>

</xml_diff>